<commit_message>
refactor(evidence): rename core evidence and clarify definition
</commit_message>
<xml_diff>
--- a/evaluation/evidence_prep_draft.xlsx
+++ b/evaluation/evidence_prep_draft.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aoyu/Library/CloudStorage/GoogleDrive-fish73078@gmail.com/我的云端硬盘/School/PolyU/Semester_02/DSAI5201_Artificial-Intelligence-and-Big-Data-Computing-in-Practice/Proj/solution/experiment/questions/for commit/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aoyu/Projects/coursework/AIP/proj/Lightweight-RAG-System-for-Academic-Papers/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E8F97A-270E-4240-A358-473543DDBEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{256E9FF5-8F85-EA48-8E0B-DDF0DB3E3602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7420" yWindow="8300" windowWidth="31360" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15200" yWindow="7820" windowWidth="31360" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Evidence Prep" sheetId="4" r:id="rId1"/>
@@ -159,12 +159,6 @@
     <t>QID</t>
   </si>
   <si>
-    <t>Gold Evidence Location (Temp)</t>
-  </si>
-  <si>
-    <t>Gold Evidence Text</t>
-  </si>
-  <si>
     <t>Supporting Evidence Location (Temp)</t>
   </si>
   <si>
@@ -759,6 +753,14 @@
   </si>
   <si>
     <t>6,7</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Core Evidence Text</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Core Evidence Location (Temp)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1053,19 +1055,19 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1" t="s">
+        <v>235</v>
+      </c>
+      <c r="F1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>43</v>
-      </c>
-      <c r="G1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1073,22 +1075,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
       </c>
       <c r="D2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" t="s">
         <v>46</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>47</v>
-      </c>
-      <c r="F2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1096,22 +1098,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
       </c>
       <c r="D3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" t="s">
         <v>50</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>51</v>
-      </c>
-      <c r="F3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1119,22 +1121,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
       </c>
       <c r="D4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" t="s">
         <v>54</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>55</v>
-      </c>
-      <c r="F4" t="s">
-        <v>56</v>
-      </c>
-      <c r="G4" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1142,22 +1144,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
       </c>
       <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" t="s">
         <v>58</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>59</v>
-      </c>
-      <c r="F5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G5" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1165,22 +1167,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
       </c>
       <c r="D6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" t="s">
         <v>62</v>
       </c>
-      <c r="E6" t="s">
+      <c r="G6" t="s">
         <v>63</v>
-      </c>
-      <c r="F6" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1188,22 +1190,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="D7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="F7" t="s">
-        <v>68</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1211,22 +1213,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="D8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="F8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1234,22 +1236,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C9" t="s">
         <v>9</v>
       </c>
       <c r="D9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" t="s">
         <v>74</v>
       </c>
-      <c r="E9" t="s">
+      <c r="G9" t="s">
         <v>75</v>
-      </c>
-      <c r="F9" t="s">
-        <v>76</v>
-      </c>
-      <c r="G9" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1257,22 +1259,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C10" t="s">
         <v>10</v>
       </c>
       <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="E10" t="s">
+      <c r="G10" t="s">
         <v>79</v>
-      </c>
-      <c r="F10" t="s">
-        <v>80</v>
-      </c>
-      <c r="G10" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1280,22 +1282,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
       </c>
       <c r="D11" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" t="s">
         <v>82</v>
       </c>
-      <c r="E11" t="s">
+      <c r="G11" t="s">
         <v>83</v>
-      </c>
-      <c r="F11" t="s">
-        <v>84</v>
-      </c>
-      <c r="G11" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1303,22 +1305,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" t="s">
         <v>86</v>
       </c>
-      <c r="E12" t="s">
+      <c r="G12" t="s">
         <v>87</v>
-      </c>
-      <c r="F12" t="s">
-        <v>88</v>
-      </c>
-      <c r="G12" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1326,22 +1328,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C13" t="s">
         <v>13</v>
       </c>
       <c r="D13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" t="s">
         <v>90</v>
       </c>
-      <c r="E13" t="s">
+      <c r="G13" t="s">
         <v>91</v>
-      </c>
-      <c r="F13" t="s">
-        <v>92</v>
-      </c>
-      <c r="G13" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1349,22 +1351,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C14" t="s">
         <v>14</v>
       </c>
       <c r="D14" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" t="s">
+        <v>93</v>
+      </c>
+      <c r="F14" t="s">
         <v>94</v>
       </c>
-      <c r="E14" t="s">
+      <c r="G14" t="s">
         <v>95</v>
-      </c>
-      <c r="F14" t="s">
-        <v>96</v>
-      </c>
-      <c r="G14" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1372,22 +1374,22 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C15" t="s">
         <v>15</v>
       </c>
       <c r="D15" t="s">
+        <v>96</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F15" t="s">
         <v>98</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="F15" t="s">
-        <v>100</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1395,22 +1397,22 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C16" t="s">
         <v>16</v>
       </c>
       <c r="D16" t="s">
+        <v>100</v>
+      </c>
+      <c r="E16" t="s">
+        <v>101</v>
+      </c>
+      <c r="F16" t="s">
         <v>102</v>
       </c>
-      <c r="E16" t="s">
+      <c r="G16" t="s">
         <v>103</v>
-      </c>
-      <c r="F16" t="s">
-        <v>104</v>
-      </c>
-      <c r="G16" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1418,22 +1420,22 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C17" t="s">
         <v>17</v>
       </c>
       <c r="D17" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17" t="s">
+        <v>105</v>
+      </c>
+      <c r="F17" t="s">
         <v>106</v>
       </c>
-      <c r="E17" t="s">
+      <c r="G17" t="s">
         <v>107</v>
-      </c>
-      <c r="F17" t="s">
-        <v>108</v>
-      </c>
-      <c r="G17" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1441,22 +1443,22 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C18" t="s">
         <v>18</v>
       </c>
       <c r="D18" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" t="s">
+        <v>109</v>
+      </c>
+      <c r="F18" t="s">
         <v>110</v>
       </c>
-      <c r="E18" t="s">
+      <c r="G18" t="s">
         <v>111</v>
-      </c>
-      <c r="F18" t="s">
-        <v>112</v>
-      </c>
-      <c r="G18" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1464,22 +1466,22 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C19" t="s">
         <v>19</v>
       </c>
       <c r="D19" t="s">
+        <v>112</v>
+      </c>
+      <c r="E19" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" t="s">
         <v>114</v>
       </c>
-      <c r="E19" t="s">
+      <c r="G19" t="s">
         <v>115</v>
-      </c>
-      <c r="F19" t="s">
-        <v>116</v>
-      </c>
-      <c r="G19" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1487,22 +1489,22 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C20" t="s">
         <v>20</v>
       </c>
       <c r="D20" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" t="s">
         <v>118</v>
       </c>
-      <c r="E20" t="s">
+      <c r="G20" t="s">
         <v>119</v>
-      </c>
-      <c r="F20" t="s">
-        <v>120</v>
-      </c>
-      <c r="G20" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1510,22 +1512,22 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C21" t="s">
         <v>21</v>
       </c>
       <c r="D21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E21" t="s">
+        <v>121</v>
+      </c>
+      <c r="F21" t="s">
         <v>122</v>
       </c>
-      <c r="E21" t="s">
+      <c r="G21" t="s">
         <v>123</v>
-      </c>
-      <c r="F21" t="s">
-        <v>124</v>
-      </c>
-      <c r="G21" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1533,22 +1535,22 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C22" t="s">
         <v>22</v>
       </c>
       <c r="D22" t="s">
+        <v>124</v>
+      </c>
+      <c r="E22" t="s">
+        <v>125</v>
+      </c>
+      <c r="F22" t="s">
         <v>126</v>
       </c>
-      <c r="E22" t="s">
+      <c r="G22" t="s">
         <v>127</v>
-      </c>
-      <c r="F22" t="s">
-        <v>128</v>
-      </c>
-      <c r="G22" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1556,22 +1558,22 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C23" t="s">
         <v>23</v>
       </c>
       <c r="D23" t="s">
+        <v>128</v>
+      </c>
+      <c r="E23" t="s">
+        <v>129</v>
+      </c>
+      <c r="F23" t="s">
         <v>130</v>
       </c>
-      <c r="E23" t="s">
+      <c r="G23" t="s">
         <v>131</v>
-      </c>
-      <c r="F23" t="s">
-        <v>132</v>
-      </c>
-      <c r="G23" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1579,22 +1581,22 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C24" t="s">
         <v>24</v>
       </c>
       <c r="D24" t="s">
+        <v>132</v>
+      </c>
+      <c r="E24" t="s">
+        <v>133</v>
+      </c>
+      <c r="F24" t="s">
         <v>134</v>
       </c>
-      <c r="E24" t="s">
+      <c r="G24" t="s">
         <v>135</v>
-      </c>
-      <c r="F24" t="s">
-        <v>136</v>
-      </c>
-      <c r="G24" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1602,22 +1604,22 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C25" t="s">
         <v>25</v>
       </c>
       <c r="D25" t="s">
+        <v>136</v>
+      </c>
+      <c r="E25" t="s">
+        <v>137</v>
+      </c>
+      <c r="F25" t="s">
         <v>138</v>
       </c>
-      <c r="E25" t="s">
+      <c r="G25" t="s">
         <v>139</v>
-      </c>
-      <c r="F25" t="s">
-        <v>140</v>
-      </c>
-      <c r="G25" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1625,22 +1627,22 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C26" t="s">
         <v>26</v>
       </c>
       <c r="D26" t="s">
+        <v>140</v>
+      </c>
+      <c r="E26" t="s">
+        <v>141</v>
+      </c>
+      <c r="F26" t="s">
         <v>142</v>
       </c>
-      <c r="E26" t="s">
+      <c r="G26" t="s">
         <v>143</v>
-      </c>
-      <c r="F26" t="s">
-        <v>144</v>
-      </c>
-      <c r="G26" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1648,22 +1650,22 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C27" t="s">
         <v>27</v>
       </c>
       <c r="D27" t="s">
+        <v>144</v>
+      </c>
+      <c r="E27" t="s">
+        <v>145</v>
+      </c>
+      <c r="F27" t="s">
         <v>146</v>
       </c>
-      <c r="E27" t="s">
+      <c r="G27" t="s">
         <v>147</v>
-      </c>
-      <c r="F27" t="s">
-        <v>148</v>
-      </c>
-      <c r="G27" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1677,16 +1679,16 @@
         <v>28</v>
       </c>
       <c r="D28" t="s">
+        <v>148</v>
+      </c>
+      <c r="E28" t="s">
+        <v>149</v>
+      </c>
+      <c r="F28" t="s">
         <v>150</v>
       </c>
-      <c r="E28" t="s">
+      <c r="G28" t="s">
         <v>151</v>
-      </c>
-      <c r="F28" t="s">
-        <v>152</v>
-      </c>
-      <c r="G28" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1700,16 +1702,16 @@
         <v>30</v>
       </c>
       <c r="D29" t="s">
+        <v>152</v>
+      </c>
+      <c r="E29" t="s">
+        <v>153</v>
+      </c>
+      <c r="F29" t="s">
         <v>154</v>
       </c>
-      <c r="E29" t="s">
+      <c r="G29" t="s">
         <v>155</v>
-      </c>
-      <c r="F29" t="s">
-        <v>156</v>
-      </c>
-      <c r="G29" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1717,22 +1719,22 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D30" t="s">
+        <v>156</v>
+      </c>
+      <c r="E30" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" t="s">
         <v>158</v>
       </c>
-      <c r="E30" t="s">
+      <c r="G30" t="s">
         <v>159</v>
-      </c>
-      <c r="F30" t="s">
-        <v>160</v>
-      </c>
-      <c r="G30" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1740,22 +1742,22 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D31" t="s">
+        <v>160</v>
+      </c>
+      <c r="E31" t="s">
+        <v>161</v>
+      </c>
+      <c r="F31" t="s">
         <v>162</v>
       </c>
-      <c r="E31" t="s">
+      <c r="G31" t="s">
         <v>163</v>
-      </c>
-      <c r="F31" t="s">
-        <v>164</v>
-      </c>
-      <c r="G31" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1763,22 +1765,22 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C32" t="s">
         <v>34</v>
       </c>
       <c r="D32" t="s">
+        <v>164</v>
+      </c>
+      <c r="E32" t="s">
+        <v>165</v>
+      </c>
+      <c r="F32" t="s">
         <v>166</v>
       </c>
-      <c r="E32" t="s">
+      <c r="G32" t="s">
         <v>167</v>
-      </c>
-      <c r="F32" t="s">
-        <v>168</v>
-      </c>
-      <c r="G32" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1786,22 +1788,22 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C33" t="s">
         <v>35</v>
       </c>
       <c r="D33" t="s">
+        <v>168</v>
+      </c>
+      <c r="E33" t="s">
+        <v>169</v>
+      </c>
+      <c r="F33" t="s">
         <v>170</v>
       </c>
-      <c r="E33" t="s">
+      <c r="G33" t="s">
         <v>171</v>
-      </c>
-      <c r="F33" t="s">
-        <v>172</v>
-      </c>
-      <c r="G33" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1809,22 +1811,22 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C34" t="s">
         <v>36</v>
       </c>
       <c r="D34" t="s">
+        <v>172</v>
+      </c>
+      <c r="E34" t="s">
+        <v>173</v>
+      </c>
+      <c r="F34" t="s">
         <v>174</v>
       </c>
-      <c r="E34" t="s">
+      <c r="G34" t="s">
         <v>175</v>
-      </c>
-      <c r="F34" t="s">
-        <v>176</v>
-      </c>
-      <c r="G34" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1832,22 +1834,22 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C35" t="s">
         <v>37</v>
       </c>
       <c r="D35" t="s">
+        <v>176</v>
+      </c>
+      <c r="E35" t="s">
+        <v>177</v>
+      </c>
+      <c r="F35" t="s">
         <v>178</v>
       </c>
-      <c r="E35" t="s">
+      <c r="G35" t="s">
         <v>179</v>
-      </c>
-      <c r="F35" t="s">
-        <v>180</v>
-      </c>
-      <c r="G35" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1855,22 +1857,22 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C36" t="s">
         <v>38</v>
       </c>
       <c r="D36" t="s">
+        <v>180</v>
+      </c>
+      <c r="E36" t="s">
+        <v>181</v>
+      </c>
+      <c r="F36" t="s">
         <v>182</v>
       </c>
-      <c r="E36" t="s">
+      <c r="G36" t="s">
         <v>183</v>
-      </c>
-      <c r="F36" t="s">
-        <v>184</v>
-      </c>
-      <c r="G36" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1878,22 +1880,22 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C37" t="s">
         <v>39</v>
       </c>
       <c r="D37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E37" t="s">
+        <v>184</v>
+      </c>
+      <c r="F37" t="s">
+        <v>185</v>
+      </c>
+      <c r="G37" t="s">
         <v>186</v>
-      </c>
-      <c r="F37" t="s">
-        <v>187</v>
-      </c>
-      <c r="G37" t="s">
-        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -1913,19 +1915,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1933,16 +1935,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C2">
         <v>2021</v>
       </c>
       <c r="D2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1950,16 +1952,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C3">
         <v>2023</v>
       </c>
       <c r="D3" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1967,16 +1969,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C4">
         <v>2024</v>
       </c>
       <c r="D4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E4" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1984,16 +1986,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C5">
         <v>2024</v>
       </c>
       <c r="D5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2001,16 +2003,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C6">
         <v>2023</v>
       </c>
       <c r="D6" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E6" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2018,16 +2020,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C7">
         <v>2023</v>
       </c>
       <c r="D7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2035,16 +2037,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C8">
         <v>2022</v>
       </c>
       <c r="D8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2052,16 +2054,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C9">
         <v>2023</v>
       </c>
       <c r="D9" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2069,16 +2071,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C10">
         <v>2024</v>
       </c>
       <c r="D10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2086,16 +2088,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C11">
         <v>2024</v>
       </c>
       <c r="D11" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>